<commit_message>
Update reviews: 26 new (2026-08-21)
</commit_message>
<xml_diff>
--- a/otzyvy_halyk.xlsx
+++ b/otzyvy_halyk.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3213,6 +3213,1154 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46253.51787037037</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>App Store</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Ужасное приложение банка</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Еле грузит, колл-центр типа с искусственными интеллектом который тупо молчит! Куда звонить!? Пишу в поддержку ответы тоже ии без решения проблемы. Вам до Каспи банка далеко!</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Злая 1479(</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>7.15.0</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>14446617149</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>46254.38908564814</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>5</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Класс!</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Laiosh Tolnai</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>a2b1475d0a4636044e411f96</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>46254.37627314815</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>5</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>очень удобно оплачивать ком услуги ну и все остальное</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Анаргуль Есенгалиева</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>0d69e28794204a7ebc123308</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>46254.37443287037</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>все хорошо. спасибо</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Кайрат Маусымхан</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>7d68f1ac71d4d9fa0e6e7239</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>46254.36811342592</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Пока всё отлично! Просто, удобно.</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Наталья Энзе</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>ebfe0c1582b6e0efd21a9304</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>46254.29225694444</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>👍👍👍</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Serikkali Moldahmetov</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>8f08456f1f7037ddfc48fb40</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>46254.26644675926</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>5</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Спасибо!Быстро и качественно.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Фарит Абдуллин</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>4bc036aaba61bf9681d0c2f8</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>46254.23796296296</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>4</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Очень удобный сервис!!!</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Камшат Есентаева</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>6ce3a6058942a3a52ea23739</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>46254.18957175926</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Рахмет очень удобно пользоваться</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Мария Кулёва</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>974572017a25b0123bd5f57c</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>46254.15381944444</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>5</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>хорошо спасибо</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Elmurat Bayanov</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>abd0fd54964a3ac6c73eaf28</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>46254.12082175926</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>люблю халык банк</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Береза График</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>6147099de51977f68610bbdc</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>46254.10601851852</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>5</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>супер</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Бахтыгуль Алдажарова</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>af62592e2b234acc94cae3c7</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>46254.0353587963</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>5</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Халык Алакан тоже сделайте, чтобы рукой можно было оплачивать</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Бауыржан Джаримбетов</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>3bf98a3770b05e9be2c430cb</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>46253.99089120371</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>5</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>отлично</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Гульмира Тащанова</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>915995320029b26e5b7f6f0a</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46253.94253472222</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>довольно часто не работает приложение</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Зарина Султанова</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>0ed11d36c4bb48b15370e5e2</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>46253.93590277778</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>5</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>очень очень приятно</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Асхат Ногайбаев</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>a4b69efb01fca2c81b220ec9</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>46253.92797453704</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>5</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>очень удобное и нужное приложение.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Adai</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>c2834899d00d38c54b8deb58</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>46253.91368055555</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>5</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>күшті</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Марат Газизович</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>4451aeedc50f456c670fa41c</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n">
+        <v>46253.91197916667</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>отличное приложение</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Kaiyrzhan Makhanov</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>534dacc61d02bb38aa52d612</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46253.89833333333</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>мало функции , те которые есть не совсем просто использовать , можно сделать проще и доступнее . Очень мало интернет магазинов ...</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Dos Dosanov</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>a4e57b2dff2e9988d2957d0d</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>46253.87689814815</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>удобно</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Aisar Atabek</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>c9e20cbacf740c765c59a66c</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>46253.85269675926</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>иногда не могу найти историю платежа в приложении. например когда оплачиваешь проезд на автобус, когда выходишь не сможешь найти, а там реклама</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Багила Берниязова</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>27532977d33acaf460206cc3</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46253.85040509259</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Ешқандай техподержка операторға хабарласақ тек обновит етіп қойдықтан басқасын аитпайды оператор сойлем аяқталмай телефонды өшіріп тастайды</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Сапармурат Абдуллаев</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>7.15.2</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>9c8033c621be3a2064bb1efc</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>46253.83737268519</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Данияр Мусаев</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>cae9951351f128d20380f025</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46253.83456018518</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>бежать нужно с этого банка</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>виталий Шабалин</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>17b166bf83abe143eadce261</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46253.77180555555</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>kz</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>пОлучать сообщения опополнении</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Живой Некромант</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>7.14.0</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>4c30970474e4542378188c99</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>